<commit_message>
update branding & rest. planning layout; .xlsx & .csv cleaning
</commit_message>
<xml_diff>
--- a/www/Baseline_Cover_EXAMPLE.xlsx
+++ b/www/Baseline_Cover_EXAMPLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640D451A-3ED0-4E94-8415-3828602DA506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6811350D-1251-4867-A7E2-81F126876BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="71895" yWindow="22140" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="4170" yWindow="3578" windowWidth="18870" windowHeight="11265" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
@@ -298,9 +298,6 @@
     <t>Percent_Cover</t>
   </si>
   <si>
-    <t>REQUIRED_Unconsolidated_substrate</t>
-  </si>
-  <si>
     <t>Cladocora arbuscula</t>
   </si>
   <si>
@@ -421,6 +418,9 @@
   </si>
   <si>
     <t>Mote_EDR10</t>
+  </si>
+  <si>
+    <t>REQUIRED Unconsolidated substrate</t>
   </si>
 </sst>
 </file>
@@ -858,22 +858,22 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
@@ -881,47 +881,47 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -976,10 +976,10 @@
         <v>83</v>
       </c>
       <c r="J1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K1" t="s">
         <v>100</v>
-      </c>
-      <c r="K1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
@@ -990,16 +990,16 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="C2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" t="s">
         <v>103</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>104</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>105</v>
-      </c>
-      <c r="F2" t="s">
-        <v>106</v>
       </c>
       <c r="G2" s="6">
         <v>24.459129999999998</v>
@@ -1011,10 +1011,10 @@
         <v>100</v>
       </c>
       <c r="J2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K2" t="s">
         <v>107</v>
-      </c>
-      <c r="K2" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
@@ -1025,16 +1025,16 @@
         <v>0.2</v>
       </c>
       <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" t="s">
         <v>103</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>104</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>105</v>
-      </c>
-      <c r="F3" t="s">
-        <v>106</v>
       </c>
       <c r="G3" s="6">
         <v>24.459129999999998</v>
@@ -1046,10 +1046,10 @@
         <v>100</v>
       </c>
       <c r="J3" t="s">
+        <v>106</v>
+      </c>
+      <c r="K3" t="s">
         <v>107</v>
-      </c>
-      <c r="K3" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
@@ -1060,16 +1060,16 @@
         <v>1.5</v>
       </c>
       <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="s">
         <v>103</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>104</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>105</v>
-      </c>
-      <c r="F4" t="s">
-        <v>106</v>
       </c>
       <c r="G4" s="6">
         <v>24.459129999999998</v>
@@ -1081,30 +1081,30 @@
         <v>100</v>
       </c>
       <c r="J4" t="s">
+        <v>106</v>
+      </c>
+      <c r="K4" t="s">
         <v>107</v>
-      </c>
-      <c r="K4" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="B5">
         <v>5</v>
       </c>
       <c r="C5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" t="s">
         <v>103</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>104</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>105</v>
-      </c>
-      <c r="F5" t="s">
-        <v>106</v>
       </c>
       <c r="G5" s="6">
         <v>24.459129999999998</v>
@@ -1116,10 +1116,10 @@
         <v>100</v>
       </c>
       <c r="J5" t="s">
+        <v>106</v>
+      </c>
+      <c r="K5" t="s">
         <v>107</v>
-      </c>
-      <c r="K5" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.45">
@@ -1130,16 +1130,16 @@
         <v>0.1</v>
       </c>
       <c r="C6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" t="s">
         <v>103</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>104</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>105</v>
-      </c>
-      <c r="F6" t="s">
-        <v>106</v>
       </c>
       <c r="G6" s="6">
         <v>24.459129999999998</v>
@@ -1151,10 +1151,10 @@
         <v>100</v>
       </c>
       <c r="J6" t="s">
+        <v>106</v>
+      </c>
+      <c r="K6" t="s">
         <v>107</v>
-      </c>
-      <c r="K6" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.45">
@@ -1165,16 +1165,16 @@
         <v>7.7</v>
       </c>
       <c r="C7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
         <v>103</v>
       </c>
-      <c r="D7" t="s">
-        <v>104</v>
-      </c>
       <c r="E7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G7" s="6">
         <v>24.45889</v>
@@ -1186,30 +1186,30 @@
         <v>100</v>
       </c>
       <c r="J7" t="s">
+        <v>106</v>
+      </c>
+      <c r="K7" t="s">
         <v>107</v>
-      </c>
-      <c r="K7" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" t="s">
         <v>103</v>
       </c>
-      <c r="D8" t="s">
-        <v>104</v>
-      </c>
       <c r="E8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G8" s="6">
         <v>24.45889</v>
@@ -1221,10 +1221,10 @@
         <v>100</v>
       </c>
       <c r="J8" t="s">
+        <v>106</v>
+      </c>
+      <c r="K8" t="s">
         <v>107</v>
-      </c>
-      <c r="K8" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.45">
@@ -1277,7 +1277,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.45">
@@ -1347,7 +1347,7 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
@@ -1522,7 +1522,7 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.45">
@@ -1677,26 +1677,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -1891,26 +1871,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1929,6 +1910,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>

<commit_message>
real outplant mortality data; timeline SLR display toggle
</commit_message>
<xml_diff>
--- a/www/Baseline_Cover_EXAMPLE.xlsx
+++ b/www/Baseline_Cover_EXAMPLE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cjenkins\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21653D09-B4DA-47E7-8014-0545E1F6F268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0D835D-72B8-4D5D-99FF-508AC86C91FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2512" yWindow="2512" windowWidth="14521" windowHeight="11333" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3188" yWindow="3188" windowWidth="14520" windowHeight="11332" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="131">
   <si>
     <t>Coral Cover Data Input README:</t>
   </si>
@@ -45,6 +45,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
       </rPr>
       <t>Step 1</t>
     </r>
@@ -53,12 +54,10 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">: Input the measured or estimated percent cover of each calcifying taxon (hard corals + crustose coralline algae) in the  "Coral Cover input" tab of this spreadsheet. </t>
     </r>
-  </si>
-  <si>
-    <t>REQUIRED_Unconsolidated_substrate</t>
   </si>
   <si>
     <r>
@@ -66,6 +65,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">• </t>
     </r>
@@ -74,6 +74,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
       </rPr>
       <t>Species names must exactly match the names listed in "Taxon list" or you will receive an error. If you copy/paste Taxon names from another data source rather than using the dropdown Taxon list, please ensure your taxon names are an exact match to those in "Taxon list"</t>
     </r>
@@ -160,6 +161,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
       </rPr>
       <t>Step 2</t>
     </r>
@@ -169,6 +171,7 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
+        <family val="2"/>
       </rPr>
       <t>: Input site metadata</t>
     </r>
@@ -494,33 +497,38 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Quattrocento Sans"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -860,12 +868,12 @@
     </row>
     <row r="3" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -873,47 +881,47 @@
     </row>
     <row r="6" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B13" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B14" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -1932,54 +1940,54 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="G1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="I1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="K1" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B2" s="2">
         <v>2.2999999999999998</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G2" s="5">
         <v>24.459129999999998</v>
@@ -1991,30 +1999,30 @@
         <v>100</v>
       </c>
       <c r="J2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B3" s="2">
         <v>0.2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G3" s="5">
         <v>24.459129999999998</v>
@@ -2026,30 +2034,30 @@
         <v>100</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B4" s="2">
         <v>1.5</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G4" s="5">
         <v>24.459129999999998</v>
@@ -2061,30 +2069,30 @@
         <v>100</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B5" s="2">
         <v>5</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="F5" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G5" s="5">
         <v>24.459129999999998</v>
@@ -2096,30 +2104,30 @@
         <v>100</v>
       </c>
       <c r="J5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K5" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="F6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G6" s="5">
         <v>24.459129999999998</v>
@@ -2131,30 +2139,30 @@
         <v>100</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2">
         <v>7.7</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G7" s="5">
         <v>24.45889</v>
@@ -2166,30 +2174,30 @@
         <v>100</v>
       </c>
       <c r="J7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B8" s="2">
         <v>2</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G8" s="5">
         <v>24.45889</v>
@@ -2201,30 +2209,30 @@
         <v>100</v>
       </c>
       <c r="J8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="G9" s="2">
         <v>24.616584899999999</v>
@@ -2238,22 +2246,22 @@
     </row>
     <row r="10" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2">
         <v>6</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="G10" s="2">
         <v>24.616584899999999</v>
@@ -2267,22 +2275,22 @@
     </row>
     <row r="11" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B11" s="2">
         <v>19</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="G11" s="2">
         <v>24.616584899999999</v>
@@ -2296,22 +2304,22 @@
     </row>
     <row r="12" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" s="2">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E12" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="G12" s="2">
         <v>25.036133329999998</v>
@@ -2325,22 +2333,22 @@
     </row>
     <row r="13" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="G13" s="2">
         <v>25.036133329999998</v>
@@ -2354,22 +2362,22 @@
     </row>
     <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E14" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="G14" s="2">
         <v>25.036133329999998</v>
@@ -2383,22 +2391,22 @@
     </row>
     <row r="15" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="2">
         <v>6.5</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="G15" s="2">
         <v>25.036133329999998</v>
@@ -2412,22 +2420,22 @@
     </row>
     <row r="16" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B16" s="2">
         <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>121</v>
       </c>
       <c r="G16" s="2">
         <v>25.036133329999998</v>
@@ -2441,22 +2449,22 @@
     </row>
     <row r="17" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17" s="2">
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="G17" s="2">
         <v>24.456499999999998</v>
@@ -2470,22 +2478,22 @@
     </row>
     <row r="18" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B18" s="2">
         <v>1.5</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E18" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F18" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="G18" s="2">
         <v>24.456499999999998</v>
@@ -2499,22 +2507,22 @@
     </row>
     <row r="19" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19" s="2">
         <v>7.5</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E19" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="G19" s="2">
         <v>24.456499999999998</v>
@@ -2528,22 +2536,22 @@
     </row>
     <row r="20" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B20" s="2">
         <v>15.5</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E20" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="G20" s="2">
         <v>24.456499999999998</v>
@@ -2557,22 +2565,22 @@
     </row>
     <row r="21" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B21" s="2">
         <v>4</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E21" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G21" s="2">
         <v>24.885100000000001</v>
@@ -2586,22 +2594,22 @@
     </row>
     <row r="22" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="2">
         <v>2</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E22" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G22" s="2">
         <v>24.885100000000001</v>
@@ -2615,22 +2623,22 @@
     </row>
     <row r="23" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B23" s="2">
         <v>2</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E23" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G23" s="2">
         <v>24.885100000000001</v>
@@ -2644,22 +2652,22 @@
     </row>
     <row r="24" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B24" s="2">
         <v>6</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E24" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G24" s="2">
         <v>24.885100000000001</v>
@@ -2673,22 +2681,22 @@
     </row>
     <row r="25" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B25" s="2">
         <v>14</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E25" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G25" s="2">
         <v>24.885100000000001</v>
@@ -2702,22 +2710,22 @@
     </row>
     <row r="26" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B26" s="2">
         <v>1</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G26" s="2">
         <v>24.910219999999999</v>
@@ -2731,22 +2739,22 @@
     </row>
     <row r="27" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B27" s="2">
         <v>1</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G27" s="2">
         <v>24.910219999999999</v>
@@ -2760,22 +2768,22 @@
     </row>
     <row r="28" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B28" s="2">
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G28" s="2">
         <v>24.910219999999999</v>
@@ -2789,22 +2797,22 @@
     </row>
     <row r="29" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="2">
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G29" s="2">
         <v>24.910219999999999</v>
@@ -2818,22 +2826,22 @@
     </row>
     <row r="30" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B30" s="2">
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E30" s="2" t="s">
+      <c r="F30" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G30" s="2">
         <v>24.910219999999999</v>
@@ -2847,22 +2855,22 @@
     </row>
     <row r="31" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B31" s="2">
         <v>2</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G31" s="2">
         <v>24.910219999999999</v>
@@ -2876,22 +2884,22 @@
     </row>
     <row r="32" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B32" s="2">
         <v>2</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G32" s="2">
         <v>24.910219999999999</v>
@@ -2905,22 +2913,22 @@
     </row>
     <row r="33" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B33" s="2">
         <v>0</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G33" s="2">
         <v>24.910219999999999</v>
@@ -2934,22 +2942,22 @@
     </row>
     <row r="34" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B34" s="2">
         <v>35</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D34" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G34" s="2">
         <v>24.910219999999999</v>
@@ -2963,22 +2971,22 @@
     </row>
     <row r="35" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" s="2">
         <v>4.5</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="G35" s="2">
         <v>25.215733329999999</v>
@@ -2992,22 +3000,22 @@
     </row>
     <row r="36" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B36" s="2">
         <v>1.5</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="F36" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="G36" s="2">
         <v>25.215733329999999</v>
@@ -3021,22 +3029,22 @@
     </row>
     <row r="37" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B37" s="2">
         <v>1.5</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D37" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="G37" s="2">
         <v>25.215733329999999</v>
@@ -3050,22 +3058,22 @@
     </row>
     <row r="38" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B38" s="2">
         <v>8.5</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D38" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="G38" s="2">
         <v>25.215733329999999</v>
@@ -3079,22 +3087,22 @@
     </row>
     <row r="39" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B39" s="2">
         <v>22.5</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D39" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="G39" s="2">
         <v>25.215733329999999</v>
@@ -3108,22 +3116,22 @@
     </row>
     <row r="40" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B40" s="2">
         <v>1</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G40" s="2">
         <v>24.934650000000001</v>
@@ -3137,22 +3145,22 @@
     </row>
     <row r="41" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B41" s="2">
         <v>6</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E41" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G41" s="2">
         <v>24.934650000000001</v>
@@ -3166,22 +3174,22 @@
     </row>
     <row r="42" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B42" s="2">
         <v>19</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E42" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G42" s="2">
         <v>24.934650000000001</v>
@@ -3195,22 +3203,22 @@
     </row>
     <row r="43" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B43" s="2">
         <v>1</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E43" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G43" s="2">
         <v>24.934650000000001</v>
@@ -3224,22 +3232,22 @@
     </row>
     <row r="44" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B44" s="2">
         <v>3.5</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G44" s="2">
         <v>24.934650000000001</v>
@@ -3253,22 +3261,22 @@
     </row>
     <row r="45" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B45" s="2">
         <v>6</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E45" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G45" s="2">
         <v>24.934650000000001</v>
@@ -3282,22 +3290,22 @@
     </row>
     <row r="46" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B46" s="2">
         <v>2</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E46" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="G46" s="2">
         <v>24.934650000000001</v>
@@ -3311,22 +3319,22 @@
     </row>
     <row r="47" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47">
         <v>7.5</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E47" t="s">
+        <v>126</v>
+      </c>
+      <c r="F47" t="s">
         <v>127</v>
-      </c>
-      <c r="F47" t="s">
-        <v>128</v>
       </c>
       <c r="G47">
         <v>24.521383329999999</v>
@@ -3340,22 +3348,22 @@
     </row>
     <row r="48" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B48">
         <v>14.5</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E48" t="s">
+        <v>126</v>
+      </c>
+      <c r="F48" t="s">
         <v>127</v>
-      </c>
-      <c r="F48" t="s">
-        <v>128</v>
       </c>
       <c r="G48">
         <v>24.521383329999999</v>
@@ -3369,22 +3377,22 @@
     </row>
     <row r="49" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B49">
         <v>4</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E49" t="s">
+        <v>126</v>
+      </c>
+      <c r="F49" t="s">
         <v>127</v>
-      </c>
-      <c r="F49" t="s">
-        <v>128</v>
       </c>
       <c r="G49">
         <v>24.521383329999999</v>
@@ -3398,22 +3406,22 @@
     </row>
     <row r="50" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B50">
         <v>1.5</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E50" t="s">
+        <v>126</v>
+      </c>
+      <c r="F50" t="s">
         <v>127</v>
-      </c>
-      <c r="F50" t="s">
-        <v>128</v>
       </c>
       <c r="G50">
         <v>24.521383329999999</v>
@@ -3427,22 +3435,22 @@
     </row>
     <row r="51" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B51">
         <v>1</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E51" t="s">
+        <v>126</v>
+      </c>
+      <c r="F51" t="s">
         <v>127</v>
-      </c>
-      <c r="F51" t="s">
-        <v>128</v>
       </c>
       <c r="G51">
         <v>24.521383329999999</v>
@@ -3456,22 +3464,22 @@
     </row>
     <row r="52" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B52">
         <v>4.5</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E52" t="s">
+        <v>126</v>
+      </c>
+      <c r="F52" t="s">
         <v>127</v>
-      </c>
-      <c r="F52" t="s">
-        <v>128</v>
       </c>
       <c r="G52">
         <v>24.521383329999999</v>
@@ -3485,22 +3493,22 @@
     </row>
     <row r="53" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B53">
         <v>4.5</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E53" t="s">
+        <v>126</v>
+      </c>
+      <c r="F53" t="s">
         <v>127</v>
-      </c>
-      <c r="F53" t="s">
-        <v>128</v>
       </c>
       <c r="G53">
         <v>24.521383329999999</v>
@@ -3514,22 +3522,22 @@
     </row>
     <row r="54" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B54">
         <v>8</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E54" t="s">
+        <v>126</v>
+      </c>
+      <c r="F54" t="s">
         <v>127</v>
-      </c>
-      <c r="F54" t="s">
-        <v>128</v>
       </c>
       <c r="G54">
         <v>24.521383329999999</v>
@@ -3543,22 +3551,22 @@
     </row>
     <row r="55" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B55">
         <v>19.5</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E55" t="s">
+        <v>126</v>
+      </c>
+      <c r="F55" t="s">
         <v>127</v>
-      </c>
-      <c r="F55" t="s">
-        <v>128</v>
       </c>
       <c r="G55">
         <v>24.521383329999999</v>
@@ -3572,22 +3580,22 @@
     </row>
     <row r="56" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B56">
         <v>4.5</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E56" t="s">
+        <v>128</v>
+      </c>
+      <c r="F56" t="s">
         <v>129</v>
-      </c>
-      <c r="F56" t="s">
-        <v>130</v>
       </c>
       <c r="G56">
         <v>24.4832</v>
@@ -3601,22 +3609,22 @@
     </row>
     <row r="57" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B57">
         <v>6</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E57" t="s">
+        <v>128</v>
+      </c>
+      <c r="F57" t="s">
         <v>129</v>
-      </c>
-      <c r="F57" t="s">
-        <v>130</v>
       </c>
       <c r="G57">
         <v>24.4832</v>
@@ -3630,22 +3638,22 @@
     </row>
     <row r="58" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B58">
         <v>1</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E58" t="s">
+        <v>128</v>
+      </c>
+      <c r="F58" t="s">
         <v>129</v>
-      </c>
-      <c r="F58" t="s">
-        <v>130</v>
       </c>
       <c r="G58">
         <v>24.4832</v>
@@ -3659,22 +3667,22 @@
     </row>
     <row r="59" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B59">
         <v>3</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E59" t="s">
+        <v>128</v>
+      </c>
+      <c r="F59" t="s">
         <v>129</v>
-      </c>
-      <c r="F59" t="s">
-        <v>130</v>
       </c>
       <c r="G59">
         <v>24.4832</v>
@@ -3688,22 +3696,22 @@
     </row>
     <row r="60" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B60">
         <v>1.5</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E60" t="s">
+        <v>128</v>
+      </c>
+      <c r="F60" t="s">
         <v>129</v>
-      </c>
-      <c r="F60" t="s">
-        <v>130</v>
       </c>
       <c r="G60">
         <v>24.4832</v>
@@ -3717,22 +3725,22 @@
     </row>
     <row r="61" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B61">
         <v>6.5</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E61" t="s">
+        <v>128</v>
+      </c>
+      <c r="F61" t="s">
         <v>129</v>
-      </c>
-      <c r="F61" t="s">
-        <v>130</v>
       </c>
       <c r="G61">
         <v>24.4832</v>
@@ -3746,22 +3754,22 @@
     </row>
     <row r="62" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B62">
         <v>3</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E62" t="s">
+        <v>128</v>
+      </c>
+      <c r="F62" t="s">
         <v>129</v>
-      </c>
-      <c r="F62" t="s">
-        <v>130</v>
       </c>
       <c r="G62">
         <v>24.4832</v>
@@ -3775,22 +3783,22 @@
     </row>
     <row r="63" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B63">
         <v>2</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E63" t="s">
+        <v>128</v>
+      </c>
+      <c r="F63" t="s">
         <v>129</v>
-      </c>
-      <c r="F63" t="s">
-        <v>130</v>
       </c>
       <c r="G63">
         <v>24.4832</v>
@@ -3804,22 +3812,22 @@
     </row>
     <row r="64" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B64">
         <v>18</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E64" t="s">
+        <v>128</v>
+      </c>
+      <c r="F64" t="s">
         <v>129</v>
-      </c>
-      <c r="F64" t="s">
-        <v>130</v>
       </c>
       <c r="G64">
         <v>24.4832</v>
@@ -8555,397 +8563,397 @@
     </row>
     <row r="2" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="47" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="51" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="52" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="54" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="55" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="56" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="58" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="59" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="61" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="62" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="63" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="64" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="65" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="66" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="67" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="68" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="69" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="72" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="73" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="74" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="75" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="76" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="77" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="78" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="79" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="80" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
add CCA diameter and growth rate; remove generalized taxa
</commit_message>
<xml_diff>
--- a/www/Baseline_Cover_EXAMPLE.xlsx
+++ b/www/Baseline_Cover_EXAMPLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0D835D-72B8-4D5D-99FF-508AC86C91FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6203238-3524-411C-9A86-AB91011EA1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3188" yWindow="3188" windowWidth="14520" windowHeight="11332" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2543" yWindow="2543" windowWidth="21600" windowHeight="11332" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="129">
   <si>
     <t>Coral Cover Data Input README:</t>
   </si>
@@ -225,30 +225,18 @@
     <t>Favia fragum</t>
   </si>
   <si>
-    <t>Hard Coral (branching)</t>
-  </si>
-  <si>
     <t xml:space="preserve">• A Unique_Site_ID is required. Please try to be as descriptive as possible (e.g., LK_AwesomePatchReef_Site148_2026). More generic site names can be included in the optional field </t>
   </si>
   <si>
-    <t>Hard Coral (encrusting)</t>
-  </si>
-  <si>
     <t>• Latitude and Longitude for the site should be entered in decimal degrees</t>
   </si>
   <si>
-    <t>Hard Coral (foliose)</t>
-  </si>
-  <si>
     <t>•  The area of the site, in m2, must be provided</t>
   </si>
   <si>
     <t>•  Please provide a point of contact (POC) first and last name and email for the baseline site data so that we can contact you with questions, if necessary</t>
   </si>
   <si>
-    <t>Hard Coral (massive)</t>
-  </si>
-  <si>
     <t>Helioseris cucullata</t>
   </si>
   <si>
@@ -478,17 +466,30 @@
   </si>
   <si>
     <t>REQUIRED Unconsolidated substrate</t>
+  </si>
+  <si>
+    <t>John Morris</t>
+  </si>
+  <si>
+    <t>john.morris@noaa.gov</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -551,19 +552,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -906,22 +908,22 @@
     </row>
     <row r="11" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B13" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B14" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -1999,15 +2001,15 @@
         <v>100</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B3" s="2">
         <v>0.2</v>
@@ -2034,15 +2036,15 @@
         <v>100</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B4" s="2">
         <v>1.5</v>
@@ -2069,15 +2071,15 @@
         <v>100</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B5" s="2">
         <v>5</v>
@@ -2104,15 +2106,15 @@
         <v>100</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B6" s="2">
         <v>0.1</v>
@@ -2139,10 +2141,10 @@
         <v>100</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -2159,7 +2161,7 @@
         <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>36</v>
@@ -2174,15 +2176,15 @@
         <v>100</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B8" s="2">
         <v>2</v>
@@ -2194,7 +2196,7 @@
         <v>33</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>36</v>
@@ -2209,15 +2211,15 @@
         <v>100</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B9" s="2">
         <v>2</v>
@@ -2226,13 +2228,13 @@
         <v>31</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G9" s="2">
         <v>24.616584899999999</v>
@@ -2242,6 +2244,12 @@
       </c>
       <c r="I9" s="2">
         <v>100</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -2255,13 +2263,13 @@
         <v>31</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G10" s="2">
         <v>24.616584899999999</v>
@@ -2272,10 +2280,16 @@
       <c r="I10" s="2">
         <v>100</v>
       </c>
+      <c r="J10" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="11" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B11" s="2">
         <v>19</v>
@@ -2284,13 +2298,13 @@
         <v>31</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G11" s="2">
         <v>24.616584899999999</v>
@@ -2300,6 +2314,12 @@
       </c>
       <c r="I11" s="2">
         <v>100</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -2310,16 +2330,16 @@
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G12" s="2">
         <v>25.036133329999998</v>
@@ -2330,25 +2350,31 @@
       <c r="I12" s="2">
         <v>100</v>
       </c>
+      <c r="J12" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="13" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B13" s="2">
         <v>1</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G13" s="2">
         <v>25.036133329999998</v>
@@ -2359,25 +2385,31 @@
       <c r="I13" s="2">
         <v>100</v>
       </c>
+      <c r="J13" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B14" s="2">
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G14" s="2">
         <v>25.036133329999998</v>
@@ -2387,6 +2419,12 @@
       </c>
       <c r="I14" s="2">
         <v>100</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -2397,16 +2435,16 @@
         <v>6.5</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G15" s="2">
         <v>25.036133329999998</v>
@@ -2417,25 +2455,31 @@
       <c r="I15" s="2">
         <v>100</v>
       </c>
+      <c r="J15" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="16" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B16" s="2">
         <v>19</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="G16" s="2">
         <v>25.036133329999998</v>
@@ -2446,8 +2490,14 @@
       <c r="I16" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J16" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>27</v>
       </c>
@@ -2461,10 +2511,10 @@
         <v>33</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G17" s="2">
         <v>24.456499999999998</v>
@@ -2475,10 +2525,16 @@
       <c r="I17" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J17" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B18" s="2">
         <v>1.5</v>
@@ -2490,10 +2546,10 @@
         <v>33</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G18" s="2">
         <v>24.456499999999998</v>
@@ -2504,8 +2560,14 @@
       <c r="I18" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J18" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>28</v>
       </c>
@@ -2519,10 +2581,10 @@
         <v>33</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G19" s="2">
         <v>24.456499999999998</v>
@@ -2533,10 +2595,16 @@
       <c r="I19" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J19" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B20" s="2">
         <v>15.5</v>
@@ -2548,10 +2616,10 @@
         <v>33</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G20" s="2">
         <v>24.456499999999998</v>
@@ -2562,8 +2630,14 @@
       <c r="I20" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="21" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J20" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>15</v>
       </c>
@@ -2571,16 +2645,16 @@
         <v>4</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G21" s="2">
         <v>24.885100000000001</v>
@@ -2591,8 +2665,14 @@
       <c r="I21" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J21" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>27</v>
       </c>
@@ -2600,16 +2680,16 @@
         <v>2</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G22" s="2">
         <v>24.885100000000001</v>
@@ -2620,25 +2700,31 @@
       <c r="I22" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J22" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B23" s="2">
         <v>2</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G23" s="2">
         <v>24.885100000000001</v>
@@ -2649,8 +2735,14 @@
       <c r="I23" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J23" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>28</v>
       </c>
@@ -2658,16 +2750,16 @@
         <v>6</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G24" s="2">
         <v>24.885100000000001</v>
@@ -2678,25 +2770,31 @@
       <c r="I24" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J24" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B25" s="2">
         <v>14</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G25" s="2">
         <v>24.885100000000001</v>
@@ -2707,8 +2805,14 @@
       <c r="I25" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J25" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>15</v>
       </c>
@@ -2716,16 +2820,16 @@
         <v>1</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G26" s="2">
         <v>24.910219999999999</v>
@@ -2736,25 +2840,31 @@
       <c r="I26" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J26" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K26" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B27" s="2">
         <v>1</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G27" s="2">
         <v>24.910219999999999</v>
@@ -2765,25 +2875,31 @@
       <c r="I27" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J27" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B28" s="2">
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G28" s="2">
         <v>24.910219999999999</v>
@@ -2794,8 +2910,14 @@
       <c r="I28" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J28" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K28" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -2803,16 +2925,16 @@
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G29" s="2">
         <v>24.910219999999999</v>
@@ -2823,25 +2945,31 @@
       <c r="I29" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J29" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K29" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B30" s="2">
         <v>1</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G30" s="2">
         <v>24.910219999999999</v>
@@ -2852,25 +2980,31 @@
       <c r="I30" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J30" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B31" s="2">
         <v>2</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G31" s="2">
         <v>24.910219999999999</v>
@@ -2881,25 +3015,31 @@
       <c r="I31" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J31" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B32" s="2">
         <v>2</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G32" s="2">
         <v>24.910219999999999</v>
@@ -2910,8 +3050,14 @@
       <c r="I32" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J32" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>28</v>
       </c>
@@ -2919,16 +3065,16 @@
         <v>0</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G33" s="2">
         <v>24.910219999999999</v>
@@ -2939,25 +3085,31 @@
       <c r="I33" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J33" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B34" s="2">
         <v>35</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G34" s="2">
         <v>24.910219999999999</v>
@@ -2968,8 +3120,14 @@
       <c r="I34" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J34" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
         <v>27</v>
       </c>
@@ -2977,16 +3135,16 @@
         <v>4.5</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G35" s="2">
         <v>25.215733329999999</v>
@@ -2997,25 +3155,31 @@
       <c r="I35" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J35" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B36" s="2">
         <v>1.5</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G36" s="2">
         <v>25.215733329999999</v>
@@ -3026,25 +3190,31 @@
       <c r="I36" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J36" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B37" s="2">
         <v>1.5</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G37" s="2">
         <v>25.215733329999999</v>
@@ -3055,8 +3225,14 @@
       <c r="I37" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J37" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>28</v>
       </c>
@@ -3064,16 +3240,16 @@
         <v>8.5</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G38" s="2">
         <v>25.215733329999999</v>
@@ -3084,25 +3260,31 @@
       <c r="I38" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J38" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B39" s="2">
         <v>22.5</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G39" s="2">
         <v>25.215733329999999</v>
@@ -3113,8 +3295,14 @@
       <c r="I39" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J39" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>32</v>
       </c>
@@ -3122,16 +3310,16 @@
         <v>1</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D40" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="G40" s="2">
         <v>24.934650000000001</v>
@@ -3142,25 +3330,31 @@
       <c r="I40" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J40" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K40" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B41" s="2">
         <v>6</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="G41" s="2">
         <v>24.934650000000001</v>
@@ -3171,25 +3365,31 @@
       <c r="I41" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="42" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J41" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B42" s="2">
         <v>19</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D42" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="G42" s="2">
         <v>24.934650000000001</v>
@@ -3200,8 +3400,14 @@
       <c r="I42" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="43" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J42" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K42" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>27</v>
       </c>
@@ -3209,16 +3415,16 @@
         <v>1</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D43" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="G43" s="2">
         <v>24.934650000000001</v>
@@ -3229,25 +3435,31 @@
       <c r="I43" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="44" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J43" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K43" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B44" s="2">
         <v>3.5</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D44" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F44" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="G44" s="2">
         <v>24.934650000000001</v>
@@ -3258,8 +3470,14 @@
       <c r="I44" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J44" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K44" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>28</v>
       </c>
@@ -3267,16 +3485,16 @@
         <v>6</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D45" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="G45" s="2">
         <v>24.934650000000001</v>
@@ -3287,25 +3505,31 @@
       <c r="I45" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J45" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K45" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B46" s="2">
         <v>2</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D46" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="G46" s="2">
         <v>24.934650000000001</v>
@@ -3316,8 +3540,14 @@
       <c r="I46" s="2">
         <v>100</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J46" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K46" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
         <v>32</v>
       </c>
@@ -3328,13 +3558,13 @@
         <v>31</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E47" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F47" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G47">
         <v>24.521383329999999</v>
@@ -3345,10 +3575,16 @@
       <c r="I47">
         <v>100</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J47" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K47" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B48">
         <v>14.5</v>
@@ -3357,13 +3593,13 @@
         <v>31</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E48" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F48" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G48">
         <v>24.521383329999999</v>
@@ -3374,10 +3610,16 @@
       <c r="I48">
         <v>100</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J48" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K48" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B49">
         <v>4</v>
@@ -3386,13 +3628,13 @@
         <v>31</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E49" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F49" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G49">
         <v>24.521383329999999</v>
@@ -3403,8 +3645,14 @@
       <c r="I49">
         <v>100</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J49" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K49" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>27</v>
       </c>
@@ -3415,13 +3663,13 @@
         <v>31</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E50" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F50" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G50">
         <v>24.521383329999999</v>
@@ -3432,10 +3680,16 @@
       <c r="I50">
         <v>100</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J50" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K50" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B51">
         <v>1</v>
@@ -3444,13 +3698,13 @@
         <v>31</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E51" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F51" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G51">
         <v>24.521383329999999</v>
@@ -3461,10 +3715,16 @@
       <c r="I51">
         <v>100</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J51" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K51" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B52">
         <v>4.5</v>
@@ -3473,13 +3733,13 @@
         <v>31</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E52" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F52" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G52">
         <v>24.521383329999999</v>
@@ -3490,10 +3750,16 @@
       <c r="I52">
         <v>100</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J52" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K52" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B53">
         <v>4.5</v>
@@ -3502,13 +3768,13 @@
         <v>31</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E53" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F53" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G53">
         <v>24.521383329999999</v>
@@ -3519,8 +3785,14 @@
       <c r="I53">
         <v>100</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J53" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K53" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>28</v>
       </c>
@@ -3531,13 +3803,13 @@
         <v>31</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E54" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F54" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G54">
         <v>24.521383329999999</v>
@@ -3548,10 +3820,16 @@
       <c r="I54">
         <v>100</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J54" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K54" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B55">
         <v>19.5</v>
@@ -3560,13 +3838,13 @@
         <v>31</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E55" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F55" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="G55">
         <v>24.521383329999999</v>
@@ -3577,8 +3855,14 @@
       <c r="I55">
         <v>100</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J55" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K55" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
         <v>32</v>
       </c>
@@ -3589,13 +3873,13 @@
         <v>31</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E56" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F56" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G56">
         <v>24.4832</v>
@@ -3606,10 +3890,16 @@
       <c r="I56">
         <v>100</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J56" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K56" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B57">
         <v>6</v>
@@ -3618,13 +3908,13 @@
         <v>31</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E57" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F57" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G57">
         <v>24.4832</v>
@@ -3635,10 +3925,16 @@
       <c r="I57">
         <v>100</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J57" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K57" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B58">
         <v>1</v>
@@ -3647,13 +3943,13 @@
         <v>31</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E58" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F58" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G58">
         <v>24.4832</v>
@@ -3664,10 +3960,16 @@
       <c r="I58">
         <v>100</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J58" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K58" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B59">
         <v>3</v>
@@ -3676,13 +3978,13 @@
         <v>31</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E59" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F59" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G59">
         <v>24.4832</v>
@@ -3693,8 +3995,14 @@
       <c r="I59">
         <v>100</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J59" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K59" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
         <v>27</v>
       </c>
@@ -3705,13 +4013,13 @@
         <v>31</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E60" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F60" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G60">
         <v>24.4832</v>
@@ -3722,10 +4030,16 @@
       <c r="I60">
         <v>100</v>
       </c>
-    </row>
-    <row r="61" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J60" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K60" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B61">
         <v>6.5</v>
@@ -3734,13 +4048,13 @@
         <v>31</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E61" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F61" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G61">
         <v>24.4832</v>
@@ -3751,10 +4065,16 @@
       <c r="I61">
         <v>100</v>
       </c>
-    </row>
-    <row r="62" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J61" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K61" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B62">
         <v>3</v>
@@ -3763,13 +4083,13 @@
         <v>31</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E62" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F62" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G62">
         <v>24.4832</v>
@@ -3780,8 +4100,14 @@
       <c r="I62">
         <v>100</v>
       </c>
-    </row>
-    <row r="63" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J62" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K62" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
         <v>28</v>
       </c>
@@ -3792,13 +4118,13 @@
         <v>31</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E63" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F63" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G63">
         <v>24.4832</v>
@@ -3809,10 +4135,16 @@
       <c r="I63">
         <v>100</v>
       </c>
-    </row>
-    <row r="64" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="J63" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K63" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B64">
         <v>18</v>
@@ -3821,13 +4153,13 @@
         <v>31</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E64" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F64" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G64">
         <v>24.4832</v>
@@ -3837,6 +4169,12 @@
       </c>
       <c r="I64">
         <v>100</v>
+      </c>
+      <c r="J64" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="K64" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8538,7 +8876,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
-            <xm:f>Taxa!$A$2:$A$80</xm:f>
+            <xm:f>Taxa!$A$2:$A$76</xm:f>
           </x14:formula1>
           <xm:sqref>A2:A8 A47:A1000</xm:sqref>
         </x14:dataValidation>
@@ -8550,7 +8888,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:A1000"/>
+  <dimension ref="A1:A996"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="26" width="8.59765625" customWidth="1"/>
@@ -8563,7 +8901,7 @@
     </row>
     <row r="2" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8673,17 +9011,17 @@
     </row>
     <row r="24" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8693,37 +9031,37 @@
     </row>
     <row r="28" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8732,28 +9070,28 @@
       </c>
     </row>
     <row r="36" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="6" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="6" t="s">
-        <v>69</v>
+      <c r="A40" s="2" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8763,22 +9101,22 @@
     </row>
     <row r="42" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8813,27 +9151,27 @@
     </row>
     <row r="52" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="54" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="55" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
-        <v>86</v>
+        <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
     </row>
     <row r="57" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8848,7 +9186,7 @@
     </row>
     <row r="59" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
-        <v>27</v>
+        <v>89</v>
       </c>
     </row>
     <row r="60" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -8898,64 +9236,48 @@
     </row>
     <row r="69" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
     </row>
     <row r="70" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="71" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="72" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="73" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="74" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A75" s="7" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A75" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="76" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A77" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A80" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="78" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="79" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="80" spans="1:1" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="81" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="82" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="83" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -9872,17 +10194,34 @@
     <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="995" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="647735499ae6baa62e6fc7f5ed3567b4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47ff4a2bf1fedf465812d90a21a07c12" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -10077,27 +10416,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{912B1377-D028-4F6B-BCA3-FAA07CA913FB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A51B496-5B66-49CD-B810-EE45484F45CB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3804F96C-D09B-4E31-9CCC-08B800905D50}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10116,25 +10454,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A51B496-5B66-49CD-B810-EE45484F45CB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{912B1377-D028-4F6B-BCA3-FAA07CA913FB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>